<commit_message>
Unify penalty systems and fix climbing bugs
- Fix penalty table: swap center/same-side weight values for natural hand directions at angle 0
- Add base grip drain per hold type (jug=1, pocket=2, undercling=2, pinch=3, edge=3, crimp=4, sloper=5)
- Add subtype grip penalties: sidepull/gaston angles +2 grip drain
- Move cross-body from pump penalty to grip penalty (+2 first, +4 consecutive)
- Static movement now negates cross-body grip penalty
- Shake/chalk actions now decrement technique cooldowns
- Reduce chalk cooldown from 5 to 1 turn
- Update tooltip with full grip breakdown

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Effect_Table_Corrected.xlsx
+++ b/Effect_Table_Corrected.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="6" documentId="11_9519DC14D3542C5EEF6418B65B322E3B3D0CB584" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B72FBC34-526E-B748-9F38-85518613C284}"/>
   <bookViews>
-    <workbookView xWindow="12160" yWindow="3340" windowWidth="19200" windowHeight="21520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2050" yWindow="690" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -179,6 +179,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -499,7 +503,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A3:G154"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="12.5" customWidth="1"/>
     <col min="3" max="3" width="14.83203125" bestFit="1" customWidth="1"/>
@@ -510,37 +514,37 @@
     <col min="10" max="10" width="53" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
@@ -563,7 +567,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -583,7 +587,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -603,7 +607,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -623,7 +627,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -643,7 +647,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -663,7 +667,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -683,7 +687,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>13</v>
       </c>
@@ -703,7 +707,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>13</v>
       </c>
@@ -723,7 +727,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>13</v>
       </c>
@@ -743,7 +747,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>13</v>
       </c>
@@ -763,7 +767,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>13</v>
       </c>
@@ -783,7 +787,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>13</v>
       </c>
@@ -803,7 +807,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>13</v>
       </c>
@@ -823,7 +827,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>13</v>
       </c>
@@ -843,7 +847,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>13</v>
       </c>
@@ -863,7 +867,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>13</v>
       </c>
@@ -883,7 +887,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>13</v>
       </c>
@@ -903,7 +907,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>13</v>
       </c>
@@ -923,7 +927,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>13</v>
       </c>
@@ -943,7 +947,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>13</v>
       </c>
@@ -963,7 +967,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>13</v>
       </c>
@@ -983,7 +987,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>13</v>
       </c>
@@ -1003,7 +1007,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
         <v>13</v>
       </c>
@@ -1023,7 +1027,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
         <v>13</v>
       </c>
@@ -1043,7 +1047,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
         <v>13</v>
       </c>
@@ -1063,7 +1067,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>13</v>
       </c>
@@ -1083,7 +1087,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>13</v>
       </c>
@@ -1103,7 +1107,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
         <v>13</v>
       </c>
@@ -1123,7 +1127,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
         <v>13</v>
       </c>
@@ -1143,7 +1147,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
         <v>13</v>
       </c>
@@ -1163,7 +1167,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
         <v>13</v>
       </c>
@@ -1183,7 +1187,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>13</v>
       </c>
@@ -1203,7 +1207,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
         <v>13</v>
       </c>
@@ -1223,7 +1227,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>13</v>
       </c>
@@ -1243,7 +1247,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
         <v>13</v>
       </c>
@@ -1263,7 +1267,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A46" t="s">
         <v>13</v>
       </c>
@@ -1283,7 +1287,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
         <v>13</v>
       </c>
@@ -1303,7 +1307,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A48" t="s">
         <v>13</v>
       </c>
@@ -1323,7 +1327,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A49" t="s">
         <v>13</v>
       </c>
@@ -1343,7 +1347,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A50" t="s">
         <v>13</v>
       </c>
@@ -1363,7 +1367,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
         <v>13</v>
       </c>
@@ -1383,7 +1387,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
         <v>13</v>
       </c>
@@ -1403,7 +1407,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
         <v>13</v>
       </c>
@@ -1423,7 +1427,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
         <v>13</v>
       </c>
@@ -1443,7 +1447,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
         <v>13</v>
       </c>
@@ -1463,7 +1467,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A56" t="s">
         <v>13</v>
       </c>
@@ -1483,7 +1487,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
         <v>13</v>
       </c>
@@ -1503,7 +1507,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A58" t="s">
         <v>13</v>
       </c>
@@ -1523,7 +1527,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A59" t="s">
         <v>27</v>
       </c>
@@ -1543,7 +1547,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A60" t="s">
         <v>27</v>
       </c>
@@ -1563,7 +1567,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A61" t="s">
         <v>27</v>
       </c>
@@ -1583,7 +1587,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A62" t="s">
         <v>27</v>
       </c>
@@ -1603,7 +1607,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A63" t="s">
         <v>27</v>
       </c>
@@ -1623,7 +1627,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A64" t="s">
         <v>27</v>
       </c>
@@ -1643,7 +1647,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A65" t="s">
         <v>27</v>
       </c>
@@ -1663,7 +1667,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A66" t="s">
         <v>27</v>
       </c>
@@ -1683,7 +1687,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A67" t="s">
         <v>27</v>
       </c>
@@ -1703,7 +1707,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A68" t="s">
         <v>27</v>
       </c>
@@ -1723,7 +1727,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A69" t="s">
         <v>27</v>
       </c>
@@ -1743,7 +1747,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A70" t="s">
         <v>27</v>
       </c>
@@ -1763,7 +1767,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A71" t="s">
         <v>27</v>
       </c>
@@ -1783,7 +1787,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A72" t="s">
         <v>27</v>
       </c>
@@ -1803,7 +1807,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A73" t="s">
         <v>27</v>
       </c>
@@ -1823,7 +1827,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A74" t="s">
         <v>27</v>
       </c>
@@ -1843,7 +1847,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A75" t="s">
         <v>27</v>
       </c>
@@ -1863,7 +1867,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A76" t="s">
         <v>27</v>
       </c>
@@ -1883,7 +1887,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A77" t="s">
         <v>27</v>
       </c>
@@ -1903,7 +1907,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A78" t="s">
         <v>27</v>
       </c>
@@ -1923,7 +1927,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A79" t="s">
         <v>27</v>
       </c>
@@ -1943,7 +1947,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A80" t="s">
         <v>27</v>
       </c>
@@ -1963,7 +1967,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A81" t="s">
         <v>27</v>
       </c>
@@ -1983,7 +1987,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A82" t="s">
         <v>27</v>
       </c>
@@ -2003,7 +2007,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A83" t="s">
         <v>27</v>
       </c>
@@ -2023,7 +2027,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A84" t="s">
         <v>27</v>
       </c>
@@ -2043,7 +2047,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A85" t="s">
         <v>27</v>
       </c>
@@ -2063,7 +2067,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A86" t="s">
         <v>27</v>
       </c>
@@ -2083,7 +2087,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A87" t="s">
         <v>27</v>
       </c>
@@ -2103,7 +2107,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A88" t="s">
         <v>27</v>
       </c>
@@ -2123,7 +2127,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A89" t="s">
         <v>27</v>
       </c>
@@ -2143,7 +2147,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A90" t="s">
         <v>27</v>
       </c>
@@ -2163,7 +2167,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A91" t="s">
         <v>27</v>
       </c>
@@ -2183,7 +2187,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A92" t="s">
         <v>27</v>
       </c>
@@ -2203,7 +2207,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A93" t="s">
         <v>27</v>
       </c>
@@ -2223,7 +2227,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A94" t="s">
         <v>27</v>
       </c>
@@ -2243,7 +2247,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A95" t="s">
         <v>27</v>
       </c>
@@ -2263,7 +2267,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A96" t="s">
         <v>27</v>
       </c>
@@ -2283,7 +2287,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A97" t="s">
         <v>27</v>
       </c>
@@ -2303,7 +2307,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A98" t="s">
         <v>27</v>
       </c>
@@ -2323,7 +2327,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A99" t="s">
         <v>27</v>
       </c>
@@ -2343,7 +2347,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A100" t="s">
         <v>27</v>
       </c>
@@ -2363,7 +2367,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A101" t="s">
         <v>27</v>
       </c>
@@ -2383,7 +2387,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A102" t="s">
         <v>27</v>
       </c>
@@ -2403,7 +2407,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A103" t="s">
         <v>27</v>
       </c>
@@ -2423,7 +2427,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A104" t="s">
         <v>27</v>
       </c>
@@ -2443,7 +2447,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A105" t="s">
         <v>27</v>
       </c>
@@ -2463,7 +2467,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A106" t="s">
         <v>27</v>
       </c>
@@ -2483,7 +2487,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A107" t="s">
         <v>32</v>
       </c>
@@ -2503,7 +2507,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A108" t="s">
         <v>32</v>
       </c>
@@ -2523,7 +2527,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A109" t="s">
         <v>32</v>
       </c>
@@ -2543,7 +2547,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A110" t="s">
         <v>32</v>
       </c>
@@ -2563,7 +2567,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A111" t="s">
         <v>32</v>
       </c>
@@ -2583,7 +2587,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A112" t="s">
         <v>32</v>
       </c>
@@ -2603,7 +2607,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A113" t="s">
         <v>32</v>
       </c>
@@ -2623,7 +2627,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A114" t="s">
         <v>32</v>
       </c>
@@ -2643,7 +2647,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A115" t="s">
         <v>32</v>
       </c>
@@ -2663,7 +2667,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A116" t="s">
         <v>32</v>
       </c>
@@ -2683,7 +2687,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A117" t="s">
         <v>32</v>
       </c>
@@ -2703,7 +2707,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A118" t="s">
         <v>32</v>
       </c>
@@ -2723,7 +2727,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A119" t="s">
         <v>32</v>
       </c>
@@ -2743,7 +2747,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A120" t="s">
         <v>32</v>
       </c>
@@ -2763,7 +2767,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A121" t="s">
         <v>32</v>
       </c>
@@ -2783,7 +2787,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A122" t="s">
         <v>32</v>
       </c>
@@ -2803,7 +2807,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A123" t="s">
         <v>32</v>
       </c>
@@ -2823,7 +2827,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A124" t="s">
         <v>32</v>
       </c>
@@ -2843,7 +2847,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A125" t="s">
         <v>32</v>
       </c>
@@ -2863,7 +2867,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A126" t="s">
         <v>32</v>
       </c>
@@ -2883,7 +2887,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A127" t="s">
         <v>32</v>
       </c>
@@ -2903,7 +2907,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A128" t="s">
         <v>32</v>
       </c>
@@ -2923,7 +2927,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A129" t="s">
         <v>32</v>
       </c>
@@ -2943,7 +2947,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A130" t="s">
         <v>32</v>
       </c>
@@ -2963,7 +2967,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A131" t="s">
         <v>32</v>
       </c>
@@ -2983,7 +2987,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A132" t="s">
         <v>32</v>
       </c>
@@ -3003,7 +3007,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A133" t="s">
         <v>32</v>
       </c>
@@ -3023,7 +3027,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A134" t="s">
         <v>32</v>
       </c>
@@ -3043,7 +3047,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A135" t="s">
         <v>32</v>
       </c>
@@ -3063,7 +3067,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A136" t="s">
         <v>32</v>
       </c>
@@ -3083,7 +3087,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A137" t="s">
         <v>32</v>
       </c>
@@ -3103,7 +3107,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A138" t="s">
         <v>32</v>
       </c>
@@ -3123,7 +3127,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A139" t="s">
         <v>32</v>
       </c>
@@ -3143,7 +3147,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A140" t="s">
         <v>32</v>
       </c>
@@ -3163,7 +3167,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A141" t="s">
         <v>32</v>
       </c>
@@ -3183,7 +3187,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A142" t="s">
         <v>32</v>
       </c>
@@ -3203,7 +3207,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A143" t="s">
         <v>32</v>
       </c>
@@ -3223,7 +3227,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A144" t="s">
         <v>32</v>
       </c>
@@ -3243,7 +3247,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A145" t="s">
         <v>32</v>
       </c>
@@ -3263,7 +3267,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A146" t="s">
         <v>32</v>
       </c>
@@ -3283,7 +3287,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A147" t="s">
         <v>32</v>
       </c>
@@ -3303,7 +3307,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A148" t="s">
         <v>32</v>
       </c>
@@ -3323,7 +3327,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A149" t="s">
         <v>32</v>
       </c>
@@ -3343,7 +3347,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A150" t="s">
         <v>32</v>
       </c>
@@ -3363,7 +3367,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A151" t="s">
         <v>32</v>
       </c>
@@ -3383,7 +3387,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A152" t="s">
         <v>32</v>
       </c>
@@ -3403,7 +3407,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A153" t="s">
         <v>32</v>
       </c>
@@ -3423,7 +3427,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A154" t="s">
         <v>32</v>
       </c>

</xml_diff>

<commit_message>
Tune penalty table, fix pump/grip mechanics
- Update 0° diagonal penalty values for balanced cross/base costs
- Make 270° up-left L-weight and 90° up-right R-weight instant falls
- Fall when pump reaches fatigued max instead of absolute max
- Chalk now fully restores grip to available max instead of flat +5

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Effect_Table_Corrected.xlsx
+++ b/Effect_Table_Corrected.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9826d72e9687af94/Documents/Game Dev/Climbing Grid Prototype/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_9519DC14D3542C5EEF6418B65B322E3B3D0CB584" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B72FBC34-526E-B748-9F38-85518613C284}"/>
+  <xr:revisionPtr revIDLastSave="37" documentId="11_9519DC14D3542C5EEF6418B65B322E3B3D0CB584" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{01026E38-9D6F-4D47-A74B-D77A693CB474}"/>
   <bookViews>
-    <workbookView xWindow="2050" yWindow="690" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="21360" yWindow="3920" windowWidth="19200" windowHeight="21520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$10:$G$10</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -179,10 +182,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -503,7 +502,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A3:G154"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.5" customWidth="1"/>
     <col min="3" max="3" width="14.83203125" bestFit="1" customWidth="1"/>
@@ -514,37 +513,37 @@
     <col min="10" max="10" width="53" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
@@ -567,12 +566,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -587,12 +586,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -607,12 +606,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -627,12 +626,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -647,12 +646,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -667,12 +666,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -687,12 +686,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>13</v>
       </c>
       <c r="B17" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C17">
         <v>45</v>
@@ -707,12 +706,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>13</v>
       </c>
       <c r="B18" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C18">
         <v>45</v>
@@ -727,12 +726,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C19">
         <v>45</v>
@@ -747,12 +746,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C20">
         <v>45</v>
@@ -767,12 +766,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C21">
         <v>45</v>
@@ -787,12 +786,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>13</v>
       </c>
       <c r="B22" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C22">
         <v>45</v>
@@ -807,12 +806,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>13</v>
       </c>
       <c r="B23" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C23">
         <v>90</v>
@@ -821,18 +820,18 @@
         <v>15</v>
       </c>
       <c r="E23" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F23" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>13</v>
       </c>
       <c r="B24" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C24">
         <v>90</v>
@@ -841,18 +840,18 @@
         <v>15</v>
       </c>
       <c r="E24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F24" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>13</v>
       </c>
       <c r="B25" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C25">
         <v>90</v>
@@ -861,18 +860,18 @@
         <v>19</v>
       </c>
       <c r="E25" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F25" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>13</v>
       </c>
       <c r="B26" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C26">
         <v>90</v>
@@ -881,18 +880,18 @@
         <v>19</v>
       </c>
       <c r="E26" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F26" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>13</v>
       </c>
       <c r="B27" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C27">
         <v>90</v>
@@ -901,18 +900,18 @@
         <v>21</v>
       </c>
       <c r="E27" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F27" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>13</v>
       </c>
       <c r="B28" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C28">
         <v>90</v>
@@ -921,18 +920,18 @@
         <v>21</v>
       </c>
       <c r="E28" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F28" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>13</v>
       </c>
       <c r="B29" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C29">
         <v>135</v>
@@ -947,12 +946,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>13</v>
       </c>
       <c r="B30" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C30">
         <v>135</v>
@@ -967,12 +966,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>13</v>
       </c>
       <c r="B31" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C31">
         <v>135</v>
@@ -987,12 +986,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>13</v>
       </c>
       <c r="B32" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C32">
         <v>135</v>
@@ -1007,12 +1006,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>13</v>
       </c>
       <c r="B33" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C33">
         <v>135</v>
@@ -1027,12 +1026,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>13</v>
       </c>
       <c r="B34" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C34">
         <v>135</v>
@@ -1047,12 +1046,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>13</v>
       </c>
       <c r="B35" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C35">
         <v>180</v>
@@ -1067,12 +1066,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>13</v>
       </c>
       <c r="B36" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C36">
         <v>180</v>
@@ -1087,12 +1086,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>13</v>
       </c>
       <c r="B37" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C37">
         <v>180</v>
@@ -1107,12 +1106,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>13</v>
       </c>
       <c r="B38" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C38">
         <v>180</v>
@@ -1127,12 +1126,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>13</v>
       </c>
       <c r="B39" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C39">
         <v>180</v>
@@ -1147,12 +1146,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>13</v>
       </c>
       <c r="B40" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C40">
         <v>180</v>
@@ -1167,12 +1166,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>13</v>
       </c>
       <c r="B41" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C41">
         <v>225</v>
@@ -1187,12 +1186,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>13</v>
       </c>
       <c r="B42" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C42">
         <v>225</v>
@@ -1207,12 +1206,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>13</v>
       </c>
       <c r="B43" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C43">
         <v>225</v>
@@ -1227,12 +1226,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>13</v>
       </c>
       <c r="B44" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C44">
         <v>225</v>
@@ -1247,12 +1246,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>13</v>
       </c>
       <c r="B45" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C45">
         <v>225</v>
@@ -1267,12 +1266,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>13</v>
       </c>
       <c r="B46" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C46">
         <v>225</v>
@@ -1287,12 +1286,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>13</v>
       </c>
       <c r="B47" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C47">
         <v>270</v>
@@ -1301,18 +1300,18 @@
         <v>15</v>
       </c>
       <c r="E47" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F47" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>13</v>
       </c>
       <c r="B48" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C48">
         <v>270</v>
@@ -1321,18 +1320,18 @@
         <v>15</v>
       </c>
       <c r="E48" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F48" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>13</v>
       </c>
       <c r="B49" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C49">
         <v>270</v>
@@ -1341,18 +1340,18 @@
         <v>19</v>
       </c>
       <c r="E49" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F49" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>13</v>
       </c>
       <c r="B50" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C50">
         <v>270</v>
@@ -1361,18 +1360,18 @@
         <v>19</v>
       </c>
       <c r="E50" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F50" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>13</v>
       </c>
       <c r="B51" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C51">
         <v>270</v>
@@ -1381,18 +1380,18 @@
         <v>21</v>
       </c>
       <c r="E51" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F51" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>13</v>
       </c>
       <c r="B52" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C52">
         <v>270</v>
@@ -1401,18 +1400,18 @@
         <v>21</v>
       </c>
       <c r="E52" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F52" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>13</v>
       </c>
       <c r="B53" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C53">
         <v>315</v>
@@ -1427,12 +1426,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>13</v>
       </c>
       <c r="B54" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C54">
         <v>315</v>
@@ -1447,12 +1446,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>13</v>
       </c>
       <c r="B55" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C55">
         <v>315</v>
@@ -1467,12 +1466,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>13</v>
       </c>
       <c r="B56" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C56">
         <v>315</v>
@@ -1487,12 +1486,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>13</v>
       </c>
       <c r="B57" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C57">
         <v>315</v>
@@ -1507,12 +1506,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>13</v>
       </c>
       <c r="B58" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C58">
         <v>315</v>
@@ -1527,12 +1526,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>27</v>
       </c>
       <c r="B59" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C59">
         <v>0</v>
@@ -1541,18 +1540,18 @@
         <v>15</v>
       </c>
       <c r="E59" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F59" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>27</v>
       </c>
       <c r="B60" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C60">
         <v>0</v>
@@ -1561,18 +1560,18 @@
         <v>15</v>
       </c>
       <c r="E60" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F60" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>27</v>
       </c>
       <c r="B61" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C61">
         <v>0</v>
@@ -1581,18 +1580,18 @@
         <v>19</v>
       </c>
       <c r="E61" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F61" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>27</v>
       </c>
       <c r="B62" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C62">
         <v>0</v>
@@ -1601,18 +1600,18 @@
         <v>19</v>
       </c>
       <c r="E62" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F62" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>27</v>
       </c>
       <c r="B63" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C63">
         <v>0</v>
@@ -1621,18 +1620,18 @@
         <v>21</v>
       </c>
       <c r="E63" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F63" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>27</v>
       </c>
       <c r="B64" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C64">
         <v>0</v>
@@ -1641,18 +1640,18 @@
         <v>21</v>
       </c>
       <c r="E64" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F64" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>27</v>
       </c>
       <c r="B65" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C65">
         <v>45</v>
@@ -1661,18 +1660,18 @@
         <v>15</v>
       </c>
       <c r="E65" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F65" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>27</v>
       </c>
       <c r="B66" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C66">
         <v>45</v>
@@ -1681,18 +1680,18 @@
         <v>15</v>
       </c>
       <c r="E66" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F66" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>27</v>
       </c>
       <c r="B67" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C67">
         <v>45</v>
@@ -1701,18 +1700,18 @@
         <v>19</v>
       </c>
       <c r="E67" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F67" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>27</v>
       </c>
       <c r="B68" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C68">
         <v>45</v>
@@ -1721,18 +1720,18 @@
         <v>19</v>
       </c>
       <c r="E68" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F68" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>27</v>
       </c>
       <c r="B69" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C69">
         <v>45</v>
@@ -1741,18 +1740,18 @@
         <v>21</v>
       </c>
       <c r="E69" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F69" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>27</v>
       </c>
       <c r="B70" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C70">
         <v>45</v>
@@ -1761,18 +1760,18 @@
         <v>21</v>
       </c>
       <c r="E70" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F70" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>27</v>
       </c>
       <c r="B71" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C71">
         <v>90</v>
@@ -1781,18 +1780,18 @@
         <v>15</v>
       </c>
       <c r="E71" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F71" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>27</v>
       </c>
       <c r="B72" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C72">
         <v>90</v>
@@ -1801,18 +1800,18 @@
         <v>15</v>
       </c>
       <c r="E72" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F72" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>27</v>
       </c>
       <c r="B73" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C73">
         <v>90</v>
@@ -1821,18 +1820,18 @@
         <v>19</v>
       </c>
       <c r="E73" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F73" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>27</v>
       </c>
       <c r="B74" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C74">
         <v>90</v>
@@ -1841,18 +1840,18 @@
         <v>19</v>
       </c>
       <c r="E74" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F74" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>27</v>
       </c>
       <c r="B75" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C75">
         <v>90</v>
@@ -1861,18 +1860,18 @@
         <v>21</v>
       </c>
       <c r="E75" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F75" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>27</v>
       </c>
       <c r="B76" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C76">
         <v>90</v>
@@ -1881,18 +1880,18 @@
         <v>21</v>
       </c>
       <c r="E76" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F76" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>27</v>
       </c>
       <c r="B77" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C77">
         <v>135</v>
@@ -1901,18 +1900,18 @@
         <v>15</v>
       </c>
       <c r="E77" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F77" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>27</v>
       </c>
       <c r="B78" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C78">
         <v>135</v>
@@ -1921,18 +1920,18 @@
         <v>15</v>
       </c>
       <c r="E78" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F78" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>27</v>
       </c>
       <c r="B79" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C79">
         <v>135</v>
@@ -1941,18 +1940,18 @@
         <v>19</v>
       </c>
       <c r="E79" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F79" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>27</v>
       </c>
       <c r="B80" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C80">
         <v>135</v>
@@ -1961,18 +1960,18 @@
         <v>19</v>
       </c>
       <c r="E80" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F80" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>27</v>
       </c>
       <c r="B81" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C81">
         <v>135</v>
@@ -1981,18 +1980,18 @@
         <v>21</v>
       </c>
       <c r="E81" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F81" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>27</v>
       </c>
       <c r="B82" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C82">
         <v>135</v>
@@ -2001,18 +2000,18 @@
         <v>21</v>
       </c>
       <c r="E82" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F82" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>27</v>
       </c>
       <c r="B83" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C83">
         <v>180</v>
@@ -2021,18 +2020,18 @@
         <v>15</v>
       </c>
       <c r="E83" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F83" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>27</v>
       </c>
       <c r="B84" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C84">
         <v>180</v>
@@ -2041,18 +2040,18 @@
         <v>15</v>
       </c>
       <c r="E84" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F84" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>27</v>
       </c>
       <c r="B85" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C85">
         <v>180</v>
@@ -2061,18 +2060,18 @@
         <v>19</v>
       </c>
       <c r="E85" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F85" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>27</v>
       </c>
       <c r="B86" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C86">
         <v>180</v>
@@ -2081,18 +2080,18 @@
         <v>19</v>
       </c>
       <c r="E86" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F86" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>27</v>
       </c>
       <c r="B87" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C87">
         <v>180</v>
@@ -2101,18 +2100,18 @@
         <v>21</v>
       </c>
       <c r="E87" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F87" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>27</v>
       </c>
       <c r="B88" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C88">
         <v>180</v>
@@ -2121,18 +2120,18 @@
         <v>21</v>
       </c>
       <c r="E88" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F88" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>27</v>
       </c>
       <c r="B89" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C89">
         <v>225</v>
@@ -2141,18 +2140,18 @@
         <v>15</v>
       </c>
       <c r="E89" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F89" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>27</v>
       </c>
       <c r="B90" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C90">
         <v>225</v>
@@ -2161,18 +2160,18 @@
         <v>15</v>
       </c>
       <c r="E90" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F90" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>27</v>
       </c>
       <c r="B91" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C91">
         <v>225</v>
@@ -2181,18 +2180,18 @@
         <v>19</v>
       </c>
       <c r="E91" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F91" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>27</v>
       </c>
       <c r="B92" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C92">
         <v>225</v>
@@ -2201,18 +2200,18 @@
         <v>19</v>
       </c>
       <c r="E92" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F92" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>27</v>
       </c>
       <c r="B93" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C93">
         <v>225</v>
@@ -2221,18 +2220,18 @@
         <v>21</v>
       </c>
       <c r="E93" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F93" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>27</v>
       </c>
       <c r="B94" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C94">
         <v>225</v>
@@ -2241,18 +2240,18 @@
         <v>21</v>
       </c>
       <c r="E94" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F94" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>27</v>
       </c>
       <c r="B95" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C95">
         <v>270</v>
@@ -2261,18 +2260,18 @@
         <v>15</v>
       </c>
       <c r="E95" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F95" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>27</v>
       </c>
       <c r="B96" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C96">
         <v>270</v>
@@ -2281,18 +2280,18 @@
         <v>15</v>
       </c>
       <c r="E96" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F96" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>27</v>
       </c>
       <c r="B97" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C97">
         <v>270</v>
@@ -2301,18 +2300,18 @@
         <v>19</v>
       </c>
       <c r="E97" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F97" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>27</v>
       </c>
       <c r="B98" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C98">
         <v>270</v>
@@ -2321,18 +2320,18 @@
         <v>19</v>
       </c>
       <c r="E98" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F98" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>27</v>
       </c>
       <c r="B99" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C99">
         <v>270</v>
@@ -2341,18 +2340,18 @@
         <v>21</v>
       </c>
       <c r="E99" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F99" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>27</v>
       </c>
       <c r="B100" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C100">
         <v>270</v>
@@ -2361,18 +2360,18 @@
         <v>21</v>
       </c>
       <c r="E100" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F100" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>27</v>
       </c>
       <c r="B101" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C101">
         <v>315</v>
@@ -2381,18 +2380,18 @@
         <v>15</v>
       </c>
       <c r="E101" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F101" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>27</v>
       </c>
       <c r="B102" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C102">
         <v>315</v>
@@ -2401,18 +2400,18 @@
         <v>15</v>
       </c>
       <c r="E102" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F102" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>27</v>
       </c>
       <c r="B103" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C103">
         <v>315</v>
@@ -2421,18 +2420,18 @@
         <v>19</v>
       </c>
       <c r="E103" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F103" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>27</v>
       </c>
       <c r="B104" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C104">
         <v>315</v>
@@ -2441,18 +2440,18 @@
         <v>19</v>
       </c>
       <c r="E104" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F104" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>27</v>
       </c>
       <c r="B105" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C105">
         <v>315</v>
@@ -2461,18 +2460,18 @@
         <v>21</v>
       </c>
       <c r="E105" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F105" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>27</v>
       </c>
       <c r="B106" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C106">
         <v>315</v>
@@ -2481,18 +2480,18 @@
         <v>21</v>
       </c>
       <c r="E106" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F106" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>32</v>
       </c>
       <c r="B107" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C107">
         <v>0</v>
@@ -2501,13 +2500,13 @@
         <v>15</v>
       </c>
       <c r="E107" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F107" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>32</v>
       </c>
@@ -2518,56 +2517,56 @@
         <v>0</v>
       </c>
       <c r="D108" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E108" t="s">
         <v>16</v>
       </c>
       <c r="F108" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>32</v>
       </c>
       <c r="B109" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C109">
         <v>0</v>
       </c>
       <c r="D109" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E109" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F109" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>32</v>
       </c>
       <c r="B110" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C110">
         <v>0</v>
       </c>
       <c r="D110" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E110" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F110" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>32</v>
       </c>
@@ -2578,21 +2577,21 @@
         <v>0</v>
       </c>
       <c r="D111" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E111" t="s">
         <v>28</v>
       </c>
       <c r="F111" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>32</v>
       </c>
       <c r="B112" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C112">
         <v>0</v>
@@ -2601,18 +2600,18 @@
         <v>21</v>
       </c>
       <c r="E112" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F112" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>32</v>
       </c>
       <c r="B113" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C113">
         <v>45</v>
@@ -2621,13 +2620,13 @@
         <v>15</v>
       </c>
       <c r="E113" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F113" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>32</v>
       </c>
@@ -2638,56 +2637,56 @@
         <v>45</v>
       </c>
       <c r="D114" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E114" t="s">
         <v>16</v>
       </c>
       <c r="F114" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>32</v>
       </c>
       <c r="B115" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C115">
         <v>45</v>
       </c>
       <c r="D115" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E115" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F115" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>32</v>
       </c>
       <c r="B116" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C116">
         <v>45</v>
       </c>
       <c r="D116" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E116" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F116" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>32</v>
       </c>
@@ -2698,21 +2697,21 @@
         <v>45</v>
       </c>
       <c r="D117" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E117" t="s">
         <v>28</v>
       </c>
       <c r="F117" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>32</v>
       </c>
       <c r="B118" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C118">
         <v>45</v>
@@ -2721,18 +2720,18 @@
         <v>21</v>
       </c>
       <c r="E118" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F118" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>32</v>
       </c>
       <c r="B119" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C119">
         <v>90</v>
@@ -2741,13 +2740,13 @@
         <v>15</v>
       </c>
       <c r="E119" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F119" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>32</v>
       </c>
@@ -2758,56 +2757,56 @@
         <v>90</v>
       </c>
       <c r="D120" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E120" t="s">
         <v>23</v>
       </c>
       <c r="F120" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>32</v>
       </c>
       <c r="B121" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C121">
         <v>90</v>
       </c>
       <c r="D121" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E121" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F121" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>32</v>
       </c>
       <c r="B122" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C122">
         <v>90</v>
       </c>
       <c r="D122" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E122" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F122" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>32</v>
       </c>
@@ -2818,21 +2817,21 @@
         <v>90</v>
       </c>
       <c r="D123" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E123" t="s">
         <v>30</v>
       </c>
       <c r="F123" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>32</v>
       </c>
       <c r="B124" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C124">
         <v>90</v>
@@ -2841,18 +2840,18 @@
         <v>21</v>
       </c>
       <c r="E124" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F124" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>32</v>
       </c>
       <c r="B125" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C125">
         <v>135</v>
@@ -2861,13 +2860,13 @@
         <v>15</v>
       </c>
       <c r="E125" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F125" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>32</v>
       </c>
@@ -2878,7 +2877,7 @@
         <v>135</v>
       </c>
       <c r="D126" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E126" t="s">
         <v>26</v>
@@ -2887,47 +2886,47 @@
         <v>20</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>32</v>
       </c>
       <c r="B127" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C127">
         <v>135</v>
       </c>
       <c r="D127" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E127" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F127" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>32</v>
       </c>
       <c r="B128" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C128">
         <v>135</v>
       </c>
       <c r="D128" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E128" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F128" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>32</v>
       </c>
@@ -2938,21 +2937,21 @@
         <v>135</v>
       </c>
       <c r="D129" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E129" t="s">
         <v>31</v>
       </c>
       <c r="F129" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>32</v>
       </c>
       <c r="B130" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C130">
         <v>135</v>
@@ -2961,18 +2960,18 @@
         <v>21</v>
       </c>
       <c r="E130" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F130" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>32</v>
       </c>
       <c r="B131" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C131">
         <v>180</v>
@@ -2981,13 +2980,13 @@
         <v>15</v>
       </c>
       <c r="E131" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F131" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>32</v>
       </c>
@@ -2998,56 +2997,56 @@
         <v>180</v>
       </c>
       <c r="D132" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E132" t="s">
         <v>26</v>
       </c>
       <c r="F132" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>32</v>
       </c>
       <c r="B133" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C133">
         <v>180</v>
       </c>
       <c r="D133" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E133" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F133" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>32</v>
       </c>
       <c r="B134" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C134">
         <v>180</v>
       </c>
       <c r="D134" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E134" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F134" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>32</v>
       </c>
@@ -3058,21 +3057,21 @@
         <v>180</v>
       </c>
       <c r="D135" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E135" t="s">
         <v>31</v>
       </c>
       <c r="F135" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>32</v>
       </c>
       <c r="B136" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C136">
         <v>180</v>
@@ -3081,18 +3080,18 @@
         <v>21</v>
       </c>
       <c r="E136" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F136" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>32</v>
       </c>
       <c r="B137" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C137">
         <v>225</v>
@@ -3101,13 +3100,13 @@
         <v>15</v>
       </c>
       <c r="E137" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F137" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>32</v>
       </c>
@@ -3118,56 +3117,56 @@
         <v>225</v>
       </c>
       <c r="D138" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E138" t="s">
         <v>26</v>
       </c>
       <c r="F138" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>32</v>
       </c>
       <c r="B139" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C139">
         <v>225</v>
       </c>
       <c r="D139" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E139" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F139" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>32</v>
       </c>
       <c r="B140" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C140">
         <v>225</v>
       </c>
       <c r="D140" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E140" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F140" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>32</v>
       </c>
@@ -3178,21 +3177,21 @@
         <v>225</v>
       </c>
       <c r="D141" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E141" t="s">
         <v>31</v>
       </c>
       <c r="F141" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>32</v>
       </c>
       <c r="B142" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C142">
         <v>225</v>
@@ -3201,18 +3200,18 @@
         <v>21</v>
       </c>
       <c r="E142" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F142" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>32</v>
       </c>
       <c r="B143" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C143">
         <v>270</v>
@@ -3221,13 +3220,13 @@
         <v>15</v>
       </c>
       <c r="E143" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F143" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>32</v>
       </c>
@@ -3238,56 +3237,56 @@
         <v>270</v>
       </c>
       <c r="D144" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E144" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F144" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>32</v>
       </c>
       <c r="B145" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C145">
         <v>270</v>
       </c>
       <c r="D145" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E145" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F145" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>32</v>
       </c>
       <c r="B146" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C146">
         <v>270</v>
       </c>
       <c r="D146" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E146" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F146" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>32</v>
       </c>
@@ -3298,21 +3297,21 @@
         <v>270</v>
       </c>
       <c r="D147" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E147" t="s">
         <v>30</v>
       </c>
       <c r="F147" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>32</v>
       </c>
       <c r="B148" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C148">
         <v>270</v>
@@ -3321,18 +3320,18 @@
         <v>21</v>
       </c>
       <c r="E148" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F148" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>32</v>
       </c>
       <c r="B149" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C149">
         <v>315</v>
@@ -3341,13 +3340,13 @@
         <v>15</v>
       </c>
       <c r="E149" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F149" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>32</v>
       </c>
@@ -3358,56 +3357,56 @@
         <v>315</v>
       </c>
       <c r="D150" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E150" t="s">
         <v>16</v>
       </c>
       <c r="F150" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>32</v>
       </c>
       <c r="B151" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C151">
         <v>315</v>
       </c>
       <c r="D151" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E151" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F151" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>32</v>
       </c>
       <c r="B152" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C152">
         <v>315</v>
       </c>
       <c r="D152" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E152" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F152" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>32</v>
       </c>
@@ -3418,21 +3417,21 @@
         <v>315</v>
       </c>
       <c r="D153" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E153" t="s">
         <v>28</v>
       </c>
       <c r="F153" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>32</v>
       </c>
       <c r="B154" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C154">
         <v>315</v>
@@ -3441,13 +3440,18 @@
         <v>21</v>
       </c>
       <c r="E154" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F154" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A10:G10" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A11:G154">
+      <sortCondition ref="A10:A154"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Rework skills to deterministic location-gated system and major cleanup
Replace multi-rank star-purchasing RNG skill system with single-rank
location-gated puzzle skills. Simplify climbing move resolver to use
penalty levels instead of raw pump costs. Remove debug logging and
dead code across all modules (~1,744 net lines removed).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Effect_Table_Corrected.xlsx
+++ b/Effect_Table_Corrected.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9826d72e9687af94/Documents/Game Dev/Climbing Grid Prototype/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_9519DC14D3542C5EEF6418B65B322E3B3D0CB584" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B72FBC34-526E-B748-9F38-85518613C284}"/>
+  <xr:revisionPtr revIDLastSave="37" documentId="11_9519DC14D3542C5EEF6418B65B322E3B3D0CB584" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{01026E38-9D6F-4D47-A74B-D77A693CB474}"/>
   <bookViews>
-    <workbookView xWindow="2050" yWindow="690" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="21360" yWindow="3920" windowWidth="19200" windowHeight="21520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$10:$G$10</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -179,10 +182,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -503,7 +502,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A3:G154"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.5" customWidth="1"/>
     <col min="3" max="3" width="14.83203125" bestFit="1" customWidth="1"/>
@@ -514,37 +513,37 @@
     <col min="10" max="10" width="53" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
@@ -567,12 +566,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -587,12 +586,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -607,12 +606,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -627,12 +626,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -647,12 +646,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -667,12 +666,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -687,12 +686,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>13</v>
       </c>
       <c r="B17" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C17">
         <v>45</v>
@@ -707,12 +706,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>13</v>
       </c>
       <c r="B18" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C18">
         <v>45</v>
@@ -727,12 +726,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C19">
         <v>45</v>
@@ -747,12 +746,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C20">
         <v>45</v>
@@ -767,12 +766,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C21">
         <v>45</v>
@@ -787,12 +786,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>13</v>
       </c>
       <c r="B22" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C22">
         <v>45</v>
@@ -807,12 +806,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>13</v>
       </c>
       <c r="B23" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C23">
         <v>90</v>
@@ -821,18 +820,18 @@
         <v>15</v>
       </c>
       <c r="E23" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F23" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>13</v>
       </c>
       <c r="B24" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C24">
         <v>90</v>
@@ -841,18 +840,18 @@
         <v>15</v>
       </c>
       <c r="E24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F24" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>13</v>
       </c>
       <c r="B25" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C25">
         <v>90</v>
@@ -861,18 +860,18 @@
         <v>19</v>
       </c>
       <c r="E25" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F25" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>13</v>
       </c>
       <c r="B26" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C26">
         <v>90</v>
@@ -881,18 +880,18 @@
         <v>19</v>
       </c>
       <c r="E26" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F26" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>13</v>
       </c>
       <c r="B27" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C27">
         <v>90</v>
@@ -901,18 +900,18 @@
         <v>21</v>
       </c>
       <c r="E27" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F27" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>13</v>
       </c>
       <c r="B28" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C28">
         <v>90</v>
@@ -921,18 +920,18 @@
         <v>21</v>
       </c>
       <c r="E28" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F28" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>13</v>
       </c>
       <c r="B29" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C29">
         <v>135</v>
@@ -947,12 +946,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>13</v>
       </c>
       <c r="B30" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C30">
         <v>135</v>
@@ -967,12 +966,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>13</v>
       </c>
       <c r="B31" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C31">
         <v>135</v>
@@ -987,12 +986,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>13</v>
       </c>
       <c r="B32" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C32">
         <v>135</v>
@@ -1007,12 +1006,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>13</v>
       </c>
       <c r="B33" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C33">
         <v>135</v>
@@ -1027,12 +1026,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>13</v>
       </c>
       <c r="B34" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C34">
         <v>135</v>
@@ -1047,12 +1046,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>13</v>
       </c>
       <c r="B35" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C35">
         <v>180</v>
@@ -1067,12 +1066,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>13</v>
       </c>
       <c r="B36" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C36">
         <v>180</v>
@@ -1087,12 +1086,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>13</v>
       </c>
       <c r="B37" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C37">
         <v>180</v>
@@ -1107,12 +1106,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>13</v>
       </c>
       <c r="B38" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C38">
         <v>180</v>
@@ -1127,12 +1126,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>13</v>
       </c>
       <c r="B39" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C39">
         <v>180</v>
@@ -1147,12 +1146,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>13</v>
       </c>
       <c r="B40" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C40">
         <v>180</v>
@@ -1167,12 +1166,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>13</v>
       </c>
       <c r="B41" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C41">
         <v>225</v>
@@ -1187,12 +1186,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>13</v>
       </c>
       <c r="B42" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C42">
         <v>225</v>
@@ -1207,12 +1206,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>13</v>
       </c>
       <c r="B43" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C43">
         <v>225</v>
@@ -1227,12 +1226,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>13</v>
       </c>
       <c r="B44" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C44">
         <v>225</v>
@@ -1247,12 +1246,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>13</v>
       </c>
       <c r="B45" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C45">
         <v>225</v>
@@ -1267,12 +1266,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>13</v>
       </c>
       <c r="B46" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C46">
         <v>225</v>
@@ -1287,12 +1286,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>13</v>
       </c>
       <c r="B47" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C47">
         <v>270</v>
@@ -1301,18 +1300,18 @@
         <v>15</v>
       </c>
       <c r="E47" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F47" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>13</v>
       </c>
       <c r="B48" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C48">
         <v>270</v>
@@ -1321,18 +1320,18 @@
         <v>15</v>
       </c>
       <c r="E48" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F48" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>13</v>
       </c>
       <c r="B49" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C49">
         <v>270</v>
@@ -1341,18 +1340,18 @@
         <v>19</v>
       </c>
       <c r="E49" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F49" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>13</v>
       </c>
       <c r="B50" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C50">
         <v>270</v>
@@ -1361,18 +1360,18 @@
         <v>19</v>
       </c>
       <c r="E50" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F50" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>13</v>
       </c>
       <c r="B51" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C51">
         <v>270</v>
@@ -1381,18 +1380,18 @@
         <v>21</v>
       </c>
       <c r="E51" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F51" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>13</v>
       </c>
       <c r="B52" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C52">
         <v>270</v>
@@ -1401,18 +1400,18 @@
         <v>21</v>
       </c>
       <c r="E52" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F52" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>13</v>
       </c>
       <c r="B53" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C53">
         <v>315</v>
@@ -1427,12 +1426,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>13</v>
       </c>
       <c r="B54" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C54">
         <v>315</v>
@@ -1447,12 +1446,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>13</v>
       </c>
       <c r="B55" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C55">
         <v>315</v>
@@ -1467,12 +1466,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>13</v>
       </c>
       <c r="B56" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C56">
         <v>315</v>
@@ -1487,12 +1486,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>13</v>
       </c>
       <c r="B57" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C57">
         <v>315</v>
@@ -1507,12 +1506,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>13</v>
       </c>
       <c r="B58" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C58">
         <v>315</v>
@@ -1527,12 +1526,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>27</v>
       </c>
       <c r="B59" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C59">
         <v>0</v>
@@ -1541,18 +1540,18 @@
         <v>15</v>
       </c>
       <c r="E59" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F59" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>27</v>
       </c>
       <c r="B60" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C60">
         <v>0</v>
@@ -1561,18 +1560,18 @@
         <v>15</v>
       </c>
       <c r="E60" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F60" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>27</v>
       </c>
       <c r="B61" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C61">
         <v>0</v>
@@ -1581,18 +1580,18 @@
         <v>19</v>
       </c>
       <c r="E61" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F61" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>27</v>
       </c>
       <c r="B62" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C62">
         <v>0</v>
@@ -1601,18 +1600,18 @@
         <v>19</v>
       </c>
       <c r="E62" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F62" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>27</v>
       </c>
       <c r="B63" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C63">
         <v>0</v>
@@ -1621,18 +1620,18 @@
         <v>21</v>
       </c>
       <c r="E63" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F63" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>27</v>
       </c>
       <c r="B64" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C64">
         <v>0</v>
@@ -1641,18 +1640,18 @@
         <v>21</v>
       </c>
       <c r="E64" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F64" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>27</v>
       </c>
       <c r="B65" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C65">
         <v>45</v>
@@ -1661,18 +1660,18 @@
         <v>15</v>
       </c>
       <c r="E65" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F65" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>27</v>
       </c>
       <c r="B66" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C66">
         <v>45</v>
@@ -1681,18 +1680,18 @@
         <v>15</v>
       </c>
       <c r="E66" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F66" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>27</v>
       </c>
       <c r="B67" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C67">
         <v>45</v>
@@ -1701,18 +1700,18 @@
         <v>19</v>
       </c>
       <c r="E67" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F67" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>27</v>
       </c>
       <c r="B68" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C68">
         <v>45</v>
@@ -1721,18 +1720,18 @@
         <v>19</v>
       </c>
       <c r="E68" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F68" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>27</v>
       </c>
       <c r="B69" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C69">
         <v>45</v>
@@ -1741,18 +1740,18 @@
         <v>21</v>
       </c>
       <c r="E69" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F69" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>27</v>
       </c>
       <c r="B70" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C70">
         <v>45</v>
@@ -1761,18 +1760,18 @@
         <v>21</v>
       </c>
       <c r="E70" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F70" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>27</v>
       </c>
       <c r="B71" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C71">
         <v>90</v>
@@ -1781,18 +1780,18 @@
         <v>15</v>
       </c>
       <c r="E71" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F71" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>27</v>
       </c>
       <c r="B72" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C72">
         <v>90</v>
@@ -1801,18 +1800,18 @@
         <v>15</v>
       </c>
       <c r="E72" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F72" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>27</v>
       </c>
       <c r="B73" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C73">
         <v>90</v>
@@ -1821,18 +1820,18 @@
         <v>19</v>
       </c>
       <c r="E73" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F73" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>27</v>
       </c>
       <c r="B74" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C74">
         <v>90</v>
@@ -1841,18 +1840,18 @@
         <v>19</v>
       </c>
       <c r="E74" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F74" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>27</v>
       </c>
       <c r="B75" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C75">
         <v>90</v>
@@ -1861,18 +1860,18 @@
         <v>21</v>
       </c>
       <c r="E75" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F75" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>27</v>
       </c>
       <c r="B76" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C76">
         <v>90</v>
@@ -1881,18 +1880,18 @@
         <v>21</v>
       </c>
       <c r="E76" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F76" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>27</v>
       </c>
       <c r="B77" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C77">
         <v>135</v>
@@ -1901,18 +1900,18 @@
         <v>15</v>
       </c>
       <c r="E77" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F77" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>27</v>
       </c>
       <c r="B78" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C78">
         <v>135</v>
@@ -1921,18 +1920,18 @@
         <v>15</v>
       </c>
       <c r="E78" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F78" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>27</v>
       </c>
       <c r="B79" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C79">
         <v>135</v>
@@ -1941,18 +1940,18 @@
         <v>19</v>
       </c>
       <c r="E79" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F79" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>27</v>
       </c>
       <c r="B80" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C80">
         <v>135</v>
@@ -1961,18 +1960,18 @@
         <v>19</v>
       </c>
       <c r="E80" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F80" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>27</v>
       </c>
       <c r="B81" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C81">
         <v>135</v>
@@ -1981,18 +1980,18 @@
         <v>21</v>
       </c>
       <c r="E81" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F81" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>27</v>
       </c>
       <c r="B82" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C82">
         <v>135</v>
@@ -2001,18 +2000,18 @@
         <v>21</v>
       </c>
       <c r="E82" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F82" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>27</v>
       </c>
       <c r="B83" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C83">
         <v>180</v>
@@ -2021,18 +2020,18 @@
         <v>15</v>
       </c>
       <c r="E83" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F83" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>27</v>
       </c>
       <c r="B84" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C84">
         <v>180</v>
@@ -2041,18 +2040,18 @@
         <v>15</v>
       </c>
       <c r="E84" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F84" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>27</v>
       </c>
       <c r="B85" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C85">
         <v>180</v>
@@ -2061,18 +2060,18 @@
         <v>19</v>
       </c>
       <c r="E85" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F85" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>27</v>
       </c>
       <c r="B86" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C86">
         <v>180</v>
@@ -2081,18 +2080,18 @@
         <v>19</v>
       </c>
       <c r="E86" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F86" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>27</v>
       </c>
       <c r="B87" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C87">
         <v>180</v>
@@ -2101,18 +2100,18 @@
         <v>21</v>
       </c>
       <c r="E87" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F87" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>27</v>
       </c>
       <c r="B88" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C88">
         <v>180</v>
@@ -2121,18 +2120,18 @@
         <v>21</v>
       </c>
       <c r="E88" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F88" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>27</v>
       </c>
       <c r="B89" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C89">
         <v>225</v>
@@ -2141,18 +2140,18 @@
         <v>15</v>
       </c>
       <c r="E89" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F89" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>27</v>
       </c>
       <c r="B90" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C90">
         <v>225</v>
@@ -2161,18 +2160,18 @@
         <v>15</v>
       </c>
       <c r="E90" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F90" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>27</v>
       </c>
       <c r="B91" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C91">
         <v>225</v>
@@ -2181,18 +2180,18 @@
         <v>19</v>
       </c>
       <c r="E91" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F91" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>27</v>
       </c>
       <c r="B92" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C92">
         <v>225</v>
@@ -2201,18 +2200,18 @@
         <v>19</v>
       </c>
       <c r="E92" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F92" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>27</v>
       </c>
       <c r="B93" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C93">
         <v>225</v>
@@ -2221,18 +2220,18 @@
         <v>21</v>
       </c>
       <c r="E93" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F93" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>27</v>
       </c>
       <c r="B94" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C94">
         <v>225</v>
@@ -2241,18 +2240,18 @@
         <v>21</v>
       </c>
       <c r="E94" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F94" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>27</v>
       </c>
       <c r="B95" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C95">
         <v>270</v>
@@ -2261,18 +2260,18 @@
         <v>15</v>
       </c>
       <c r="E95" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F95" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>27</v>
       </c>
       <c r="B96" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C96">
         <v>270</v>
@@ -2281,18 +2280,18 @@
         <v>15</v>
       </c>
       <c r="E96" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F96" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>27</v>
       </c>
       <c r="B97" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C97">
         <v>270</v>
@@ -2301,18 +2300,18 @@
         <v>19</v>
       </c>
       <c r="E97" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F97" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>27</v>
       </c>
       <c r="B98" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C98">
         <v>270</v>
@@ -2321,18 +2320,18 @@
         <v>19</v>
       </c>
       <c r="E98" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F98" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>27</v>
       </c>
       <c r="B99" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C99">
         <v>270</v>
@@ -2341,18 +2340,18 @@
         <v>21</v>
       </c>
       <c r="E99" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F99" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>27</v>
       </c>
       <c r="B100" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C100">
         <v>270</v>
@@ -2361,18 +2360,18 @@
         <v>21</v>
       </c>
       <c r="E100" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F100" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>27</v>
       </c>
       <c r="B101" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C101">
         <v>315</v>
@@ -2381,18 +2380,18 @@
         <v>15</v>
       </c>
       <c r="E101" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F101" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>27</v>
       </c>
       <c r="B102" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C102">
         <v>315</v>
@@ -2401,18 +2400,18 @@
         <v>15</v>
       </c>
       <c r="E102" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F102" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>27</v>
       </c>
       <c r="B103" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C103">
         <v>315</v>
@@ -2421,18 +2420,18 @@
         <v>19</v>
       </c>
       <c r="E103" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F103" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>27</v>
       </c>
       <c r="B104" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C104">
         <v>315</v>
@@ -2441,18 +2440,18 @@
         <v>19</v>
       </c>
       <c r="E104" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F104" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>27</v>
       </c>
       <c r="B105" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C105">
         <v>315</v>
@@ -2461,18 +2460,18 @@
         <v>21</v>
       </c>
       <c r="E105" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F105" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>27</v>
       </c>
       <c r="B106" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C106">
         <v>315</v>
@@ -2481,18 +2480,18 @@
         <v>21</v>
       </c>
       <c r="E106" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F106" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>32</v>
       </c>
       <c r="B107" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C107">
         <v>0</v>
@@ -2501,13 +2500,13 @@
         <v>15</v>
       </c>
       <c r="E107" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F107" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>32</v>
       </c>
@@ -2518,56 +2517,56 @@
         <v>0</v>
       </c>
       <c r="D108" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E108" t="s">
         <v>16</v>
       </c>
       <c r="F108" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>32</v>
       </c>
       <c r="B109" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C109">
         <v>0</v>
       </c>
       <c r="D109" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E109" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F109" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>32</v>
       </c>
       <c r="B110" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C110">
         <v>0</v>
       </c>
       <c r="D110" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E110" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F110" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>32</v>
       </c>
@@ -2578,21 +2577,21 @@
         <v>0</v>
       </c>
       <c r="D111" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E111" t="s">
         <v>28</v>
       </c>
       <c r="F111" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>32</v>
       </c>
       <c r="B112" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C112">
         <v>0</v>
@@ -2601,18 +2600,18 @@
         <v>21</v>
       </c>
       <c r="E112" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F112" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>32</v>
       </c>
       <c r="B113" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C113">
         <v>45</v>
@@ -2621,13 +2620,13 @@
         <v>15</v>
       </c>
       <c r="E113" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F113" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>32</v>
       </c>
@@ -2638,56 +2637,56 @@
         <v>45</v>
       </c>
       <c r="D114" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E114" t="s">
         <v>16</v>
       </c>
       <c r="F114" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>32</v>
       </c>
       <c r="B115" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C115">
         <v>45</v>
       </c>
       <c r="D115" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E115" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F115" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>32</v>
       </c>
       <c r="B116" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C116">
         <v>45</v>
       </c>
       <c r="D116" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E116" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F116" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>32</v>
       </c>
@@ -2698,21 +2697,21 @@
         <v>45</v>
       </c>
       <c r="D117" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E117" t="s">
         <v>28</v>
       </c>
       <c r="F117" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>32</v>
       </c>
       <c r="B118" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C118">
         <v>45</v>
@@ -2721,18 +2720,18 @@
         <v>21</v>
       </c>
       <c r="E118" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F118" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>32</v>
       </c>
       <c r="B119" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C119">
         <v>90</v>
@@ -2741,13 +2740,13 @@
         <v>15</v>
       </c>
       <c r="E119" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F119" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>32</v>
       </c>
@@ -2758,56 +2757,56 @@
         <v>90</v>
       </c>
       <c r="D120" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E120" t="s">
         <v>23</v>
       </c>
       <c r="F120" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>32</v>
       </c>
       <c r="B121" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C121">
         <v>90</v>
       </c>
       <c r="D121" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E121" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F121" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>32</v>
       </c>
       <c r="B122" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C122">
         <v>90</v>
       </c>
       <c r="D122" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E122" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F122" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>32</v>
       </c>
@@ -2818,21 +2817,21 @@
         <v>90</v>
       </c>
       <c r="D123" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E123" t="s">
         <v>30</v>
       </c>
       <c r="F123" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>32</v>
       </c>
       <c r="B124" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C124">
         <v>90</v>
@@ -2841,18 +2840,18 @@
         <v>21</v>
       </c>
       <c r="E124" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F124" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>32</v>
       </c>
       <c r="B125" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C125">
         <v>135</v>
@@ -2861,13 +2860,13 @@
         <v>15</v>
       </c>
       <c r="E125" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F125" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>32</v>
       </c>
@@ -2878,7 +2877,7 @@
         <v>135</v>
       </c>
       <c r="D126" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E126" t="s">
         <v>26</v>
@@ -2887,47 +2886,47 @@
         <v>20</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>32</v>
       </c>
       <c r="B127" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C127">
         <v>135</v>
       </c>
       <c r="D127" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E127" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F127" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>32</v>
       </c>
       <c r="B128" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C128">
         <v>135</v>
       </c>
       <c r="D128" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E128" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F128" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>32</v>
       </c>
@@ -2938,21 +2937,21 @@
         <v>135</v>
       </c>
       <c r="D129" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E129" t="s">
         <v>31</v>
       </c>
       <c r="F129" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>32</v>
       </c>
       <c r="B130" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C130">
         <v>135</v>
@@ -2961,18 +2960,18 @@
         <v>21</v>
       </c>
       <c r="E130" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F130" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>32</v>
       </c>
       <c r="B131" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C131">
         <v>180</v>
@@ -2981,13 +2980,13 @@
         <v>15</v>
       </c>
       <c r="E131" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F131" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>32</v>
       </c>
@@ -2998,56 +2997,56 @@
         <v>180</v>
       </c>
       <c r="D132" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E132" t="s">
         <v>26</v>
       </c>
       <c r="F132" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>32</v>
       </c>
       <c r="B133" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C133">
         <v>180</v>
       </c>
       <c r="D133" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E133" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F133" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>32</v>
       </c>
       <c r="B134" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C134">
         <v>180</v>
       </c>
       <c r="D134" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E134" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F134" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>32</v>
       </c>
@@ -3058,21 +3057,21 @@
         <v>180</v>
       </c>
       <c r="D135" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E135" t="s">
         <v>31</v>
       </c>
       <c r="F135" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>32</v>
       </c>
       <c r="B136" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C136">
         <v>180</v>
@@ -3081,18 +3080,18 @@
         <v>21</v>
       </c>
       <c r="E136" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F136" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>32</v>
       </c>
       <c r="B137" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C137">
         <v>225</v>
@@ -3101,13 +3100,13 @@
         <v>15</v>
       </c>
       <c r="E137" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F137" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>32</v>
       </c>
@@ -3118,56 +3117,56 @@
         <v>225</v>
       </c>
       <c r="D138" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E138" t="s">
         <v>26</v>
       </c>
       <c r="F138" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>32</v>
       </c>
       <c r="B139" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C139">
         <v>225</v>
       </c>
       <c r="D139" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E139" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F139" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>32</v>
       </c>
       <c r="B140" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C140">
         <v>225</v>
       </c>
       <c r="D140" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E140" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F140" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>32</v>
       </c>
@@ -3178,21 +3177,21 @@
         <v>225</v>
       </c>
       <c r="D141" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E141" t="s">
         <v>31</v>
       </c>
       <c r="F141" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>32</v>
       </c>
       <c r="B142" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C142">
         <v>225</v>
@@ -3201,18 +3200,18 @@
         <v>21</v>
       </c>
       <c r="E142" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F142" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>32</v>
       </c>
       <c r="B143" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C143">
         <v>270</v>
@@ -3221,13 +3220,13 @@
         <v>15</v>
       </c>
       <c r="E143" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F143" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>32</v>
       </c>
@@ -3238,56 +3237,56 @@
         <v>270</v>
       </c>
       <c r="D144" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E144" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F144" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>32</v>
       </c>
       <c r="B145" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C145">
         <v>270</v>
       </c>
       <c r="D145" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E145" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F145" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>32</v>
       </c>
       <c r="B146" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C146">
         <v>270</v>
       </c>
       <c r="D146" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E146" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F146" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>32</v>
       </c>
@@ -3298,21 +3297,21 @@
         <v>270</v>
       </c>
       <c r="D147" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E147" t="s">
         <v>30</v>
       </c>
       <c r="F147" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>32</v>
       </c>
       <c r="B148" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C148">
         <v>270</v>
@@ -3321,18 +3320,18 @@
         <v>21</v>
       </c>
       <c r="E148" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F148" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>32</v>
       </c>
       <c r="B149" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C149">
         <v>315</v>
@@ -3341,13 +3340,13 @@
         <v>15</v>
       </c>
       <c r="E149" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F149" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>32</v>
       </c>
@@ -3358,56 +3357,56 @@
         <v>315</v>
       </c>
       <c r="D150" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E150" t="s">
         <v>16</v>
       </c>
       <c r="F150" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>32</v>
       </c>
       <c r="B151" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C151">
         <v>315</v>
       </c>
       <c r="D151" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E151" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F151" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>32</v>
       </c>
       <c r="B152" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C152">
         <v>315</v>
       </c>
       <c r="D152" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E152" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F152" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>32</v>
       </c>
@@ -3418,21 +3417,21 @@
         <v>315</v>
       </c>
       <c r="D153" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E153" t="s">
         <v>28</v>
       </c>
       <c r="F153" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>32</v>
       </c>
       <c r="B154" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C154">
         <v>315</v>
@@ -3441,13 +3440,18 @@
         <v>21</v>
       </c>
       <c r="E154" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F154" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A10:G10" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A11:G154">
+      <sortCondition ref="A10:A154"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Split route data into per-area files and update design docs
- Extract all route definitions from routes-data.js into separate js/routes-area0..7.js files, keeping routes-data.js as the penalty table and assembly hub
- Add CLAUDE.md with project context and coding conventions
- Rename and add area2 routes: new 'The Weight', renamed 'Show You The Weigh' and 'Don't Fall A Weigh'
- Revise game design.md with updated area/route structure and skill teaching plan
- Remove outdated docs: MODIFIERS_NEW_SYSTEM.md, legacy-skills-archive.md, puzzle-climbing-system-prompt.md, Route List.xlsx
- Update route-editor penalty-data, simulator, solver, and editor to match current system
- Minor tweaks to area0 route txt files and ui-tooltip

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Effect_Table_Corrected.xlsx
+++ b/Effect_Table_Corrected.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9826d72e9687af94/Documents/Game Dev/Climbing Grid Prototype/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="37" documentId="11_9519DC14D3542C5EEF6418B65B322E3B3D0CB584" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{01026E38-9D6F-4D47-A74B-D77A693CB474}"/>
+  <xr:revisionPtr revIDLastSave="45" documentId="11_9519DC14D3542C5EEF6418B65B322E3B3D0CB584" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84658FF5-8E78-4FB6-AB65-1AE9DD67BC21}"/>
   <bookViews>
-    <workbookView xWindow="21360" yWindow="3920" windowWidth="19200" windowHeight="21520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25425" yWindow="2505" windowWidth="21420" windowHeight="18390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$10:$G$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$10:$G$154</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="34">
   <si>
     <t>If we say a hold can be angled only at 45 degree increments, here are the ideal weight positions to incur the least penalties</t>
   </si>
@@ -122,6 +122,9 @@
   </si>
   <si>
     <t>Up 1 Right 1</t>
+  </si>
+  <si>
+    <t>Sidepull, Cross</t>
   </si>
 </sst>
 </file>
@@ -501,49 +504,50 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A3:G154"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.5" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="34.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="34.375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="53" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
@@ -566,7 +570,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -586,7 +590,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -606,7 +610,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -626,7 +630,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -646,7 +650,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -666,7 +670,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -686,7 +690,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>13</v>
       </c>
@@ -706,7 +710,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>13</v>
       </c>
@@ -726,7 +730,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>13</v>
       </c>
@@ -746,7 +750,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>13</v>
       </c>
@@ -766,7 +770,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>13</v>
       </c>
@@ -786,7 +790,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>13</v>
       </c>
@@ -806,7 +810,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>13</v>
       </c>
@@ -826,7 +830,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>13</v>
       </c>
@@ -846,7 +850,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>13</v>
       </c>
@@ -866,7 +870,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>13</v>
       </c>
@@ -886,7 +890,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>13</v>
       </c>
@@ -906,7 +910,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>13</v>
       </c>
@@ -926,7 +930,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>13</v>
       </c>
@@ -946,7 +950,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>13</v>
       </c>
@@ -966,7 +970,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>13</v>
       </c>
@@ -986,7 +990,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>13</v>
       </c>
@@ -1006,7 +1010,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>13</v>
       </c>
@@ -1026,7 +1030,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>13</v>
       </c>
@@ -1046,7 +1050,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>13</v>
       </c>
@@ -1066,7 +1070,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>13</v>
       </c>
@@ -1086,7 +1090,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>13</v>
       </c>
@@ -1106,7 +1110,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>13</v>
       </c>
@@ -1126,7 +1130,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>13</v>
       </c>
@@ -1146,7 +1150,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>13</v>
       </c>
@@ -1166,7 +1170,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>13</v>
       </c>
@@ -1186,7 +1190,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>13</v>
       </c>
@@ -1206,7 +1210,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>13</v>
       </c>
@@ -1226,7 +1230,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>13</v>
       </c>
@@ -1246,7 +1250,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>13</v>
       </c>
@@ -1266,7 +1270,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>13</v>
       </c>
@@ -1286,7 +1290,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>13</v>
       </c>
@@ -1306,7 +1310,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>13</v>
       </c>
@@ -1326,7 +1330,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>13</v>
       </c>
@@ -1346,7 +1350,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>13</v>
       </c>
@@ -1366,7 +1370,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>13</v>
       </c>
@@ -1386,7 +1390,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>13</v>
       </c>
@@ -1406,7 +1410,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>13</v>
       </c>
@@ -1426,7 +1430,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>13</v>
       </c>
@@ -1446,7 +1450,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>13</v>
       </c>
@@ -1466,7 +1470,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>13</v>
       </c>
@@ -1486,7 +1490,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>13</v>
       </c>
@@ -1506,7 +1510,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>13</v>
       </c>
@@ -1526,7 +1530,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>27</v>
       </c>
@@ -1546,7 +1550,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>27</v>
       </c>
@@ -1566,7 +1570,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>27</v>
       </c>
@@ -1586,7 +1590,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>27</v>
       </c>
@@ -1606,7 +1610,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>27</v>
       </c>
@@ -1626,7 +1630,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>27</v>
       </c>
@@ -1646,7 +1650,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>27</v>
       </c>
@@ -1666,7 +1670,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>27</v>
       </c>
@@ -1686,7 +1690,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>27</v>
       </c>
@@ -1706,7 +1710,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>27</v>
       </c>
@@ -1726,7 +1730,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>27</v>
       </c>
@@ -1746,7 +1750,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>27</v>
       </c>
@@ -1766,7 +1770,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>27</v>
       </c>
@@ -1780,13 +1784,13 @@
         <v>15</v>
       </c>
       <c r="E71" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F71" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>27</v>
       </c>
@@ -1800,13 +1804,13 @@
         <v>15</v>
       </c>
       <c r="E72" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="F72" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>27</v>
       </c>
@@ -1820,13 +1824,13 @@
         <v>19</v>
       </c>
       <c r="E73" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F73" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>27</v>
       </c>
@@ -1840,13 +1844,13 @@
         <v>19</v>
       </c>
       <c r="E74" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="F74" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>27</v>
       </c>
@@ -1866,7 +1870,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>27</v>
       </c>
@@ -1880,13 +1884,13 @@
         <v>21</v>
       </c>
       <c r="E76" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="F76" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>27</v>
       </c>
@@ -1906,7 +1910,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>27</v>
       </c>
@@ -1926,7 +1930,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>27</v>
       </c>
@@ -1946,7 +1950,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>27</v>
       </c>
@@ -1966,7 +1970,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>27</v>
       </c>
@@ -1986,7 +1990,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>27</v>
       </c>
@@ -2006,7 +2010,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>27</v>
       </c>
@@ -2026,7 +2030,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>27</v>
       </c>
@@ -2046,7 +2050,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>27</v>
       </c>
@@ -2066,7 +2070,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>27</v>
       </c>
@@ -2086,7 +2090,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>27</v>
       </c>
@@ -2106,7 +2110,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>27</v>
       </c>
@@ -2126,7 +2130,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>27</v>
       </c>
@@ -2146,7 +2150,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>27</v>
       </c>
@@ -2166,7 +2170,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>27</v>
       </c>
@@ -2186,7 +2190,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>27</v>
       </c>
@@ -2206,7 +2210,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>27</v>
       </c>
@@ -2226,7 +2230,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>27</v>
       </c>
@@ -2246,7 +2250,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>27</v>
       </c>
@@ -2266,7 +2270,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>27</v>
       </c>
@@ -2286,7 +2290,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>27</v>
       </c>
@@ -2306,7 +2310,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>27</v>
       </c>
@@ -2326,7 +2330,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>27</v>
       </c>
@@ -2346,7 +2350,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>27</v>
       </c>
@@ -2366,7 +2370,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>27</v>
       </c>
@@ -2386,7 +2390,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>27</v>
       </c>
@@ -2406,7 +2410,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>27</v>
       </c>
@@ -2426,7 +2430,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>27</v>
       </c>
@@ -2446,7 +2450,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>27</v>
       </c>
@@ -2466,7 +2470,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>27</v>
       </c>
@@ -2486,7 +2490,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>32</v>
       </c>
@@ -2506,7 +2510,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>32</v>
       </c>
@@ -2526,7 +2530,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>32</v>
       </c>
@@ -2546,7 +2550,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>32</v>
       </c>
@@ -2566,7 +2570,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>32</v>
       </c>
@@ -2586,7 +2590,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>32</v>
       </c>
@@ -2606,7 +2610,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>32</v>
       </c>
@@ -2626,7 +2630,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>32</v>
       </c>
@@ -2646,7 +2650,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>32</v>
       </c>
@@ -2666,7 +2670,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>32</v>
       </c>
@@ -2686,7 +2690,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>32</v>
       </c>
@@ -2706,7 +2710,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>32</v>
       </c>
@@ -2726,7 +2730,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>32</v>
       </c>
@@ -2746,7 +2750,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>32</v>
       </c>
@@ -2766,7 +2770,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>32</v>
       </c>
@@ -2786,7 +2790,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>32</v>
       </c>
@@ -2806,7 +2810,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>32</v>
       </c>
@@ -2826,7 +2830,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>32</v>
       </c>
@@ -2846,7 +2850,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>32</v>
       </c>
@@ -2866,7 +2870,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>32</v>
       </c>
@@ -2886,7 +2890,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>32</v>
       </c>
@@ -2906,7 +2910,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>32</v>
       </c>
@@ -2926,7 +2930,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>32</v>
       </c>
@@ -2946,7 +2950,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>32</v>
       </c>
@@ -2966,7 +2970,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>32</v>
       </c>
@@ -2986,7 +2990,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>32</v>
       </c>
@@ -3006,7 +3010,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>32</v>
       </c>
@@ -3026,7 +3030,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>32</v>
       </c>
@@ -3046,7 +3050,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>32</v>
       </c>
@@ -3066,7 +3070,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>32</v>
       </c>
@@ -3086,7 +3090,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>32</v>
       </c>
@@ -3106,7 +3110,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>32</v>
       </c>
@@ -3126,7 +3130,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>32</v>
       </c>
@@ -3146,7 +3150,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>32</v>
       </c>
@@ -3166,7 +3170,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>32</v>
       </c>
@@ -3186,7 +3190,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>32</v>
       </c>
@@ -3206,7 +3210,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>32</v>
       </c>
@@ -3226,7 +3230,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>32</v>
       </c>
@@ -3246,7 +3250,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>32</v>
       </c>
@@ -3266,7 +3270,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>32</v>
       </c>
@@ -3286,7 +3290,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>32</v>
       </c>
@@ -3306,7 +3310,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>32</v>
       </c>
@@ -3326,7 +3330,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>32</v>
       </c>
@@ -3346,7 +3350,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>32</v>
       </c>
@@ -3366,7 +3370,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>32</v>
       </c>
@@ -3386,7 +3390,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>32</v>
       </c>
@@ -3406,7 +3410,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>32</v>
       </c>
@@ -3426,7 +3430,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>32</v>
       </c>
@@ -3447,7 +3451,14 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A10:G10" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <autoFilter ref="A10:G154" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="4">
+      <filters>
+        <filter val="Gaston"/>
+        <filter val="Gaston, Cross"/>
+        <filter val="Sidepull"/>
+      </filters>
+    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A11:G154">
       <sortCondition ref="A10:A154"/>
     </sortState>

</xml_diff>

<commit_message>
Swap pump/grip mechanics and update area0 routes
- Grip now accumulates from hold angle/weight mismatch (penalty table); shake restores pump, chalk restores grip
- Pump now accumulates from hold type (tick-based); bars updated to reflect new direction (pump fills up, grip drains)
- Deadpoint: justShook blocks pump decay, justChalked blocks grip state change
- Area 0 routes 2 and 3 replaced with handcrafted Shake and Chalk routes
- Cross unlocks after all area 0 routes completed; Reach moves to area 1, unlocks after 2 routes
- Add routeCount skill trigger type; remove deprecated completion/areaUnlock for cross/reach
- Route text files reorganized (old bg/cc/oa names archived, new numbered names added)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Effect_Table_Corrected.xlsx
+++ b/Effect_Table_Corrected.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9826d72e9687af94/Documents/Game Dev/Climbing Grid Prototype/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="45" documentId="11_9519DC14D3542C5EEF6418B65B322E3B3D0CB584" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84658FF5-8E78-4FB6-AB65-1AE9DD67BC21}"/>
+  <xr:revisionPtr revIDLastSave="47" documentId="11_9519DC14D3542C5EEF6418B65B322E3B3D0CB584" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A4AD13F-B270-3D46-8D4C-A50ECC4B915D}"/>
   <bookViews>
-    <workbookView xWindow="25425" yWindow="2505" windowWidth="21420" windowHeight="18390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25420" yWindow="2500" windowWidth="21420" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -56,9 +56,6 @@
   </si>
   <si>
     <t>Hold subtype</t>
-  </si>
-  <si>
-    <t>Then pump/grip effect is</t>
   </si>
   <si>
     <t>Because</t>
@@ -126,6 +123,9 @@
   <si>
     <t>Sidepull, Cross</t>
   </si>
+  <si>
+    <t>Then grip effect is</t>
+  </si>
 </sst>
 </file>
 
@@ -185,6 +185,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -504,50 +508,49 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A3:G154"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.5" customWidth="1"/>
-    <col min="3" max="3" width="14.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="34.375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="34.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="53" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
@@ -564,2901 +567,2894 @@
         <v>10</v>
       </c>
       <c r="F10" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G10" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G10" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C11">
         <v>0</v>
       </c>
       <c r="D11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E11" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" t="s">
         <v>16</v>
       </c>
-      <c r="F11" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C12">
         <v>0</v>
       </c>
       <c r="D12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E12" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" t="s">
         <v>16</v>
       </c>
-      <c r="F12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C13">
         <v>0</v>
       </c>
       <c r="D13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F13" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C14">
         <v>0</v>
       </c>
       <c r="D14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F14" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C15">
         <v>0</v>
       </c>
       <c r="D15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F15" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C16">
         <v>0</v>
       </c>
       <c r="D16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F16" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C17">
         <v>45</v>
       </c>
       <c r="D17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E17" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F17" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B18" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C18">
         <v>45</v>
       </c>
       <c r="D18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E18" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F18" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C19">
         <v>45</v>
       </c>
       <c r="D19" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F19" t="s">
         <v>16</v>
       </c>
-      <c r="F19" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C20">
         <v>45</v>
       </c>
       <c r="D20" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E20" t="s">
+        <v>15</v>
+      </c>
+      <c r="F20" t="s">
         <v>16</v>
       </c>
-      <c r="F20" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B21" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C21">
         <v>45</v>
       </c>
       <c r="D21" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E21" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F21" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B22" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C22">
         <v>45</v>
       </c>
       <c r="D22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E22" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F22" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B23" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C23">
         <v>90</v>
       </c>
       <c r="D23" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F23" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B24" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C24">
         <v>90</v>
       </c>
       <c r="D24" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E24" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F24" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C25">
         <v>90</v>
       </c>
       <c r="D25" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E25" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F25" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B26" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C26">
         <v>90</v>
       </c>
       <c r="D26" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E26" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F26" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B27" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C27">
         <v>90</v>
       </c>
       <c r="D27" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E27" t="s">
+        <v>23</v>
+      </c>
+      <c r="F27" t="s">
         <v>24</v>
       </c>
-      <c r="F27" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B28" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C28">
         <v>90</v>
       </c>
       <c r="D28" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E28" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F28" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B29" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C29">
         <v>135</v>
       </c>
       <c r="D29" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E29" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F29" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B30" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C30">
         <v>135</v>
       </c>
       <c r="D30" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E30" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F30" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B31" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C31">
         <v>135</v>
       </c>
       <c r="D31" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E31" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F31" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B32" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C32">
         <v>135</v>
       </c>
       <c r="D32" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E32" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F32" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B33" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C33">
         <v>135</v>
       </c>
       <c r="D33" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E33" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F33" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B34" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C34">
         <v>135</v>
       </c>
       <c r="D34" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E34" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F34" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B35" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C35">
         <v>180</v>
       </c>
       <c r="D35" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E35" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F35" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B36" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C36">
         <v>180</v>
       </c>
       <c r="D36" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E36" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F36" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B37" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C37">
         <v>180</v>
       </c>
       <c r="D37" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E37" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F37" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B38" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C38">
         <v>180</v>
       </c>
       <c r="D38" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E38" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F38" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B39" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C39">
         <v>180</v>
       </c>
       <c r="D39" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E39" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F39" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B40" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C40">
         <v>180</v>
       </c>
       <c r="D40" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E40" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F40" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B41" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C41">
         <v>225</v>
       </c>
       <c r="D41" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E41" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F41" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B42" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C42">
         <v>225</v>
       </c>
       <c r="D42" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E42" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F42" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B43" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C43">
         <v>225</v>
       </c>
       <c r="D43" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E43" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F43" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B44" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C44">
         <v>225</v>
       </c>
       <c r="D44" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E44" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F44" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B45" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C45">
         <v>225</v>
       </c>
       <c r="D45" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E45" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F45" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B46" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C46">
         <v>225</v>
       </c>
       <c r="D46" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E46" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F46" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B47" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C47">
         <v>270</v>
       </c>
       <c r="D47" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E47" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F47" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B48" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C48">
         <v>270</v>
       </c>
       <c r="D48" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E48" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F48" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B49" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C49">
         <v>270</v>
       </c>
       <c r="D49" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E49" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F49" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B50" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C50">
         <v>270</v>
       </c>
       <c r="D50" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E50" t="s">
+        <v>23</v>
+      </c>
+      <c r="F50" t="s">
         <v>24</v>
       </c>
-      <c r="F50" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B51" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C51">
         <v>270</v>
       </c>
       <c r="D51" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E51" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F51" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B52" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C52">
         <v>270</v>
       </c>
       <c r="D52" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E52" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F52" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B53" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C53">
         <v>315</v>
       </c>
       <c r="D53" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E53" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F53" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B54" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C54">
         <v>315</v>
       </c>
       <c r="D54" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E54" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F54" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B55" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C55">
         <v>315</v>
       </c>
       <c r="D55" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E55" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F55" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B56" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C56">
         <v>315</v>
       </c>
       <c r="D56" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E56" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F56" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B57" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C57">
         <v>315</v>
       </c>
       <c r="D57" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E57" t="s">
+        <v>15</v>
+      </c>
+      <c r="F57" t="s">
         <v>16</v>
       </c>
-      <c r="F57" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B58" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C58">
         <v>315</v>
       </c>
       <c r="D58" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E58" t="s">
+        <v>15</v>
+      </c>
+      <c r="F58" t="s">
         <v>16</v>
       </c>
-      <c r="F58" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B59" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C59">
         <v>0</v>
       </c>
       <c r="D59" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E59" t="s">
+        <v>15</v>
+      </c>
+      <c r="F59" t="s">
         <v>16</v>
       </c>
-      <c r="F59" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B60" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C60">
         <v>0</v>
       </c>
       <c r="D60" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E60" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F60" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B61" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C61">
         <v>0</v>
       </c>
       <c r="D61" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E61" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F61" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B62" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C62">
         <v>0</v>
       </c>
       <c r="D62" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E62" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F62" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B63" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C63">
         <v>0</v>
       </c>
       <c r="D63" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E63" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F63" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B64" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C64">
         <v>0</v>
       </c>
       <c r="D64" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E64" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F64" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B65" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C65">
         <v>45</v>
       </c>
       <c r="D65" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E65" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F65" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B66" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C66">
         <v>45</v>
       </c>
       <c r="D66" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E66" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F66" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B67" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C67">
         <v>45</v>
       </c>
       <c r="D67" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E67" t="s">
+        <v>15</v>
+      </c>
+      <c r="F67" t="s">
         <v>16</v>
       </c>
-      <c r="F67" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B68" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C68">
         <v>45</v>
       </c>
       <c r="D68" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E68" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F68" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B69" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C69">
         <v>45</v>
       </c>
       <c r="D69" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E69" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F69" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B70" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C70">
         <v>45</v>
       </c>
       <c r="D70" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E70" t="s">
+        <v>27</v>
+      </c>
+      <c r="F70" t="s">
         <v>28</v>
       </c>
-      <c r="F70" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B71" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C71">
         <v>90</v>
       </c>
       <c r="D71" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E71" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F71" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B72" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C72">
         <v>90</v>
       </c>
       <c r="D72" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E72" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F72" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B73" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C73">
         <v>90</v>
       </c>
       <c r="D73" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E73" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F73" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B74" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C74">
         <v>90</v>
       </c>
       <c r="D74" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E74" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F74" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B75" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C75">
         <v>90</v>
       </c>
       <c r="D75" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E75" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F75" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B76" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C76">
         <v>90</v>
       </c>
       <c r="D76" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E76" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F76" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B77" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C77">
         <v>135</v>
       </c>
       <c r="D77" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E77" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F77" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B78" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C78">
         <v>135</v>
       </c>
       <c r="D78" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E78" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F78" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B79" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C79">
         <v>135</v>
       </c>
       <c r="D79" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E79" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F79" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B80" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C80">
         <v>135</v>
       </c>
       <c r="D80" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E80" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F80" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B81" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C81">
         <v>135</v>
       </c>
       <c r="D81" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E81" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F81" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B82" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C82">
         <v>135</v>
       </c>
       <c r="D82" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E82" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F82" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B83" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C83">
         <v>180</v>
       </c>
       <c r="D83" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E83" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F83" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B84" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C84">
         <v>180</v>
       </c>
       <c r="D84" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E84" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F84" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B85" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C85">
         <v>180</v>
       </c>
       <c r="D85" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E85" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F85" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B86" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C86">
         <v>180</v>
       </c>
       <c r="D86" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E86" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F86" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B87" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C87">
         <v>180</v>
       </c>
       <c r="D87" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E87" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F87" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B88" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C88">
         <v>180</v>
       </c>
       <c r="D88" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E88" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F88" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B89" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C89">
         <v>225</v>
       </c>
       <c r="D89" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E89" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F89" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B90" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C90">
         <v>225</v>
       </c>
       <c r="D90" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E90" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F90" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B91" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C91">
         <v>225</v>
       </c>
       <c r="D91" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E91" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F91" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="92" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B92" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C92">
         <v>225</v>
       </c>
       <c r="D92" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E92" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F92" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B93" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C93">
         <v>225</v>
       </c>
       <c r="D93" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E93" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F93" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B94" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C94">
         <v>225</v>
       </c>
       <c r="D94" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E94" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F94" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B95" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C95">
         <v>270</v>
       </c>
       <c r="D95" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E95" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F95" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B96" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C96">
         <v>270</v>
       </c>
       <c r="D96" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E96" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F96" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B97" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C97">
         <v>270</v>
       </c>
       <c r="D97" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E97" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F97" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B98" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C98">
         <v>270</v>
       </c>
       <c r="D98" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E98" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F98" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B99" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C99">
         <v>270</v>
       </c>
       <c r="D99" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E99" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F99" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B100" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C100">
         <v>270</v>
       </c>
       <c r="D100" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E100" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F100" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="101" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B101" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C101">
         <v>315</v>
       </c>
       <c r="D101" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E101" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F101" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="102" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B102" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C102">
         <v>315</v>
       </c>
       <c r="D102" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E102" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F102" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B103" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C103">
         <v>315</v>
       </c>
       <c r="D103" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E103" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F103" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B104" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C104">
         <v>315</v>
       </c>
       <c r="D104" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E104" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F104" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B105" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C105">
         <v>315</v>
       </c>
       <c r="D105" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E105" t="s">
+        <v>15</v>
+      </c>
+      <c r="F105" t="s">
         <v>16</v>
       </c>
-      <c r="F105" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="106" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B106" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C106">
         <v>315</v>
       </c>
       <c r="D106" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E106" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F106" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="107" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B107" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C107">
         <v>0</v>
       </c>
       <c r="D107" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E107" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F107" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B108" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C108">
         <v>0</v>
       </c>
       <c r="D108" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E108" t="s">
+        <v>15</v>
+      </c>
+      <c r="F108" t="s">
         <v>16</v>
       </c>
-      <c r="F108" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="109" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B109" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C109">
         <v>0</v>
       </c>
       <c r="D109" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E109" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F109" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B110" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C110">
         <v>0</v>
       </c>
       <c r="D110" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E110" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F110" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="111" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B111" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C111">
         <v>0</v>
       </c>
       <c r="D111" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E111" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F111" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="112" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B112" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C112">
         <v>0</v>
       </c>
       <c r="D112" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E112" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F112" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B113" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C113">
         <v>45</v>
       </c>
       <c r="D113" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E113" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F113" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="114" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B114" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C114">
         <v>45</v>
       </c>
       <c r="D114" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E114" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F114" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="115" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B115" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C115">
         <v>45</v>
       </c>
       <c r="D115" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E115" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F115" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="116" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B116" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C116">
         <v>45</v>
       </c>
       <c r="D116" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E116" t="s">
+        <v>15</v>
+      </c>
+      <c r="F116" t="s">
         <v>16</v>
       </c>
-      <c r="F116" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="117" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B117" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C117">
         <v>45</v>
       </c>
       <c r="D117" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E117" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F117" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="118" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B118" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C118">
         <v>45</v>
       </c>
       <c r="D118" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E118" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F118" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B119" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C119">
         <v>90</v>
       </c>
       <c r="D119" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E119" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F119" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B120" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C120">
         <v>90</v>
       </c>
       <c r="D120" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E120" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F120" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B121" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C121">
         <v>90</v>
       </c>
       <c r="D121" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E121" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F121" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B122" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C122">
         <v>90</v>
       </c>
       <c r="D122" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E122" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F122" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B123" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C123">
         <v>90</v>
       </c>
       <c r="D123" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E123" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F123" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B124" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C124">
         <v>90</v>
       </c>
       <c r="D124" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E124" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F124" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="125" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B125" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C125">
         <v>135</v>
       </c>
       <c r="D125" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E125" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F125" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="126" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B126" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C126">
         <v>135</v>
       </c>
       <c r="D126" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E126" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F126" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="127" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B127" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C127">
         <v>135</v>
       </c>
       <c r="D127" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E127" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F127" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="128" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B128" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C128">
         <v>135</v>
       </c>
       <c r="D128" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E128" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F128" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="129" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B129" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C129">
         <v>135</v>
       </c>
       <c r="D129" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E129" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F129" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="130" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B130" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C130">
         <v>135</v>
       </c>
       <c r="D130" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E130" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F130" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="131" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B131" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C131">
         <v>180</v>
       </c>
       <c r="D131" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E131" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F131" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="132" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B132" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C132">
         <v>180</v>
       </c>
       <c r="D132" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E132" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F132" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="133" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B133" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C133">
         <v>180</v>
       </c>
       <c r="D133" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E133" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F133" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="134" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B134" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C134">
         <v>180</v>
       </c>
       <c r="D134" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E134" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F134" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="135" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B135" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C135">
         <v>180</v>
       </c>
       <c r="D135" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E135" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F135" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="136" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B136" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C136">
         <v>180</v>
       </c>
       <c r="D136" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E136" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F136" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="137" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B137" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C137">
         <v>225</v>
       </c>
       <c r="D137" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E137" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F137" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="138" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B138" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C138">
         <v>225</v>
       </c>
       <c r="D138" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E138" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F138" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="139" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B139" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C139">
         <v>225</v>
       </c>
       <c r="D139" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E139" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F139" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="140" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B140" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C140">
         <v>225</v>
       </c>
       <c r="D140" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E140" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F140" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="141" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B141" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C141">
         <v>225</v>
       </c>
       <c r="D141" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E141" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F141" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="142" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B142" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C142">
         <v>225</v>
       </c>
       <c r="D142" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E142" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F142" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B143" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C143">
         <v>270</v>
       </c>
       <c r="D143" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E143" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F143" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B144" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C144">
         <v>270</v>
       </c>
       <c r="D144" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E144" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F144" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B145" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C145">
         <v>270</v>
       </c>
       <c r="D145" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E145" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F145" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B146" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C146">
         <v>270</v>
       </c>
       <c r="D146" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E146" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F146" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B147" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C147">
         <v>270</v>
       </c>
       <c r="D147" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E147" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F147" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B148" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C148">
         <v>270</v>
       </c>
       <c r="D148" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E148" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F148" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="149" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B149" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C149">
         <v>315</v>
       </c>
       <c r="D149" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E149" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F149" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="150" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B150" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C150">
         <v>315</v>
       </c>
       <c r="D150" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E150" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F150" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="151" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B151" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C151">
         <v>315</v>
       </c>
       <c r="D151" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E151" t="s">
+        <v>27</v>
+      </c>
+      <c r="F151" t="s">
         <v>28</v>
       </c>
-      <c r="F151" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="152" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B152" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C152">
         <v>315</v>
       </c>
       <c r="D152" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E152" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F152" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="153" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B153" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C153">
         <v>315</v>
       </c>
       <c r="D153" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E153" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F153" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="154" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B154" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C154">
         <v>315</v>
       </c>
       <c r="D154" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E154" t="s">
+        <v>15</v>
+      </c>
+      <c r="F154" t="s">
         <v>16</v>
-      </c>
-      <c r="F154" t="s">
-        <v>17</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A10:G154" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="Gaston"/>
-        <filter val="Gaston, Cross"/>
-        <filter val="Sidepull"/>
-      </filters>
-    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A11:G154">
       <sortCondition ref="A10:A154"/>
     </sortState>

</xml_diff>